<commit_message>
updated to java8 and thread document
</commit_message>
<xml_diff>
--- a/Lookup.xlsx
+++ b/Lookup.xlsx
@@ -4,19 +4,19 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tech Stack" sheetId="1" r:id="rId1"/>
     <sheet name="Interview Questions" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="interview schdule" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>NextJS</t>
   </si>
@@ -76,13 +76,47 @@
   </si>
   <si>
     <t>https://javatechonline.com/elasticsearch-with-spring-boot-spring-data-elasticsearch-crud-examples/</t>
+  </si>
+  <si>
+    <t>https://teams.microsoft.com/light-meetings/launch?context=%7B%22Tid%22%3A%22111483dd-9e03-417d-bd28-5866c2dddaa5%22%2C%22Oid%22%3A%22bb3d7561-ba4a-4aca-b493-be9c0bf07d02%22%7D&amp;anon=true&amp;lightExperience=true&amp;correlationId=24cf8bdb-ddf3-49af-82e4-00405fcb1c1f&amp;agent=web&amp;version=25101311601&amp;coords=eyJjb252ZXJzYXRpb25JZCI6IjE5Om1lZXRpbmdfT0dGaFptRXlaVFV0TlRCbFpTMDBOMkkwTFdFeU5HUXRZamhsWmpRellXTmlZakkzQHRocmVhZC52MiIsInRlbmFudElkIjoiMTExNDgzZGQtOWUwMy00MTdkLWJkMjgtNTg2NmMyZGRkYWE1Iiwib3JnYW5pemVySWQiOiJiYjNkNzU2MS1iYTRhLTRhY2EtYjQ5My1iZTljMGJmMDdkMDIiLCJtZXNzYWdlSWQiOiIwIn0%3D&amp;deeplinkId=1c009563-9659-4583-a4be-dff2b4b69114</t>
+  </si>
+  <si>
+    <t>Mobily</t>
+  </si>
+  <si>
+    <r>
+      <t>Meeting ID: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color rgb="FF242424"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>397 773 642 094 5</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Passcode: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color rgb="FF242424"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>q88Uk659</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -97,6 +131,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF616161"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF242424"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -144,13 +190,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -591,9 +639,37 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A3:A8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="99" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="17" x14ac:dyDescent="0.5">
+      <c r="A6" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="17" x14ac:dyDescent="0.5">
+      <c r="A8" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" display="https://teams.microsoft.com/light-meetings/launch?context=%7B%22Tid%22%3A%22111483dd-9e03-417d-bd28-5866c2dddaa5%22%2C%22Oid%22%3A%22bb3d7561-ba4a-4aca-b493-be9c0bf07d02%22%7D&amp;anon=true&amp;lightExperience=true&amp;correlationId=24cf8bdb-ddf3-49af-82e4-00405fcb1c"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
New Images added to docs
</commit_message>
<xml_diff>
--- a/Lookup.xlsx
+++ b/Lookup.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>NextJS</t>
   </si>
@@ -86,6 +86,60 @@
   </si>
   <si>
     <t>Jmeter.</t>
+  </si>
+  <si>
+    <t>Holder class Bill Pugh Method. Correct.</t>
+  </si>
+  <si>
+    <t>Enum singleton</t>
+  </si>
+  <si>
+    <t>Edge cases using Double check locking.</t>
+  </si>
+  <si>
+    <t>readResolve method 12</t>
+  </si>
+  <si>
+    <t>what is thread safe and synchronization.</t>
+  </si>
+  <si>
+    <t>Object pooling.</t>
+  </si>
+  <si>
+    <t>how HTTTP Request header contains</t>
+  </si>
+  <si>
+    <t>saga Orchestrator - pattern</t>
+  </si>
+  <si>
+    <t>1. Strategy Pattern</t>
+  </si>
+  <si>
+    <t>2. Observer Pattern</t>
+  </si>
+  <si>
+    <t>3. Command Pattern</t>
+  </si>
+  <si>
+    <t>4. Chain of Responsibility</t>
+  </si>
+  <si>
+    <t>5. State Pattern</t>
+  </si>
+  <si>
+    <t>6. Template Method</t>
+  </si>
+  <si>
+    <t>7. Mediator Pattern</t>
+  </si>
+  <si>
+    <t>8. Iterator Pattern</t>
+  </si>
+  <si>
+    <t>9. Memento Pattern</t>
+  </si>
+  <si>
+    <t>10. Visitor Pattern</t>
   </si>
 </sst>
 </file>
@@ -470,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="91.7265625" customWidth="1"/>
@@ -597,6 +651,101 @@
         <v>22</v>
       </c>
     </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A26" r:id="rId1"/>

</xml_diff>

<commit_message>
Some files are updated.
</commit_message>
<xml_diff>
--- a/Lookup.xlsx
+++ b/Lookup.xlsx
@@ -4,17 +4,18 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8020"/>
   </bookViews>
   <sheets>
     <sheet name="Tech Stack" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>NextJS</t>
   </si>
@@ -76,77 +77,80 @@
     <t>Magicfor kida</t>
   </si>
   <si>
-    <t>Core java+ Programmming on new features + DS + Design patterns + db concepts+ sql + Hibernate.</t>
-  </si>
-  <si>
-    <t>React js + typescript+java script</t>
-  </si>
-  <si>
     <t>spring + spring boot +Microservices + kafka</t>
   </si>
   <si>
     <t>Jmeter.</t>
   </si>
   <si>
-    <t>Holder class Bill Pugh Method. Correct.</t>
-  </si>
-  <si>
-    <t>Enum singleton</t>
-  </si>
-  <si>
-    <t>Edge cases using Double check locking.</t>
-  </si>
-  <si>
-    <t>readResolve method 12</t>
-  </si>
-  <si>
-    <t>what is thread safe and synchronization.</t>
-  </si>
-  <si>
-    <t>Object pooling.</t>
-  </si>
-  <si>
-    <t>how HTTTP Request header contains</t>
-  </si>
-  <si>
     <t>saga Orchestrator - pattern</t>
   </si>
   <si>
-    <t>1. Strategy Pattern</t>
-  </si>
-  <si>
-    <t>2. Observer Pattern</t>
-  </si>
-  <si>
-    <t>3. Command Pattern</t>
-  </si>
-  <si>
-    <t>4. Chain of Responsibility</t>
-  </si>
-  <si>
-    <t>5. State Pattern</t>
-  </si>
-  <si>
-    <t>6. Template Method</t>
-  </si>
-  <si>
-    <t>7. Mediator Pattern</t>
-  </si>
-  <si>
-    <t>8. Iterator Pattern</t>
-  </si>
-  <si>
-    <t>9. Memento Pattern</t>
-  </si>
-  <si>
-    <t>10. Visitor Pattern</t>
+    <t>Core java+ Programmming on new features + DS + Design patterns + DB Concepts + sql + Hibernate.</t>
+  </si>
+  <si>
+    <t>React js + typescript + java script</t>
+  </si>
+  <si>
+    <t>Does anyone offer paid, on-demand architect-level support for Java and Spring Boot microservices, covering system design, scalability, performance, and best practices?”</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>https://www.flipkart.com/hikvision-ezviz-c6n-wifi-indoor-smart-pan-tilt-night-vision-wireless-security-camera/p/itm6a06aa8fa0745?pid=HSAGBBXSQ6ABGUCC&amp;lid=LSTHSAGBBXSQ6ABGUCCZ5YEDC&amp;marketplace=FLIPKART&amp;cmpid=content_home-security-camera_8965229628_gmc&amp;affExtParam1=YT3-43Zi0Ddj1i5R50PxbifL8-0ysWzcOjF1hLOOgzy8RaV_uLJqDDU_Bi5iLxK2IwQliCtJWt9dbfGBMcql6rtmtpy_&amp;affid=ytflipkart</t>
+  </si>
+  <si>
+    <t>https://www.flipkart.com/accutrust-smart-visual-ear-wax-cleaner-5mp-hd-camera-wifi-connectivity-electric/p/itm0315faef11f13?pid=EECHGXCWFRH6XZHA&amp;lid=LSTEECHGXCWFRH6XZHAISPLFA&amp;marketplace=FLIPKART&amp;cmpid=content_electric-ear-cleaner_8965229628_gmc&amp;affExtParam1=YT3-z2rvmWPrOgxlKmfc_aEoLuOMgI-j9wjho2LRdfrZUYxb7nMHeUixAxq1wdbLmpADGix8YWLsz2ErZwLHghUe8bs&amp;affid=ytflipkart</t>
+  </si>
+  <si>
+    <t>Print all permutations of a string in Java</t>
+  </si>
+  <si>
+    <t>BPMS</t>
+  </si>
+  <si>
+    <r>
+      <t>Share an example of how you have taken a real-world customer problem and converted it into a scalable technical framework or reusable solution.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FFD8372A"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>*</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Summarize any complex integration project you have designed and implemented, highlighting the architecture, challenges you faced, and how you resolved them.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FFD8372A"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>*</t>
+    </r>
+  </si>
+  <si>
+    <t>Interview Questions</t>
+  </si>
+  <si>
+    <t>AWS Certification.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,6 +165,20 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <color rgb="FF282525"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <color rgb="FFD8372A"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -208,7 +226,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -216,6 +234,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -524,10 +546,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="91.7265625" customWidth="1"/>
+    <col min="1" max="1" width="91.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -602,7 +624,12 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
@@ -638,119 +665,88 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51" s="7" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A26" r:id="rId1"/>
+    <hyperlink ref="A51" r:id="rId2" display="https://www.geeksforgeeks.org/dsa/print-all-permutations-of-a-string-in-java/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="96.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update on aws tab
</commit_message>
<xml_diff>
--- a/Lookup.xlsx
+++ b/Lookup.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80A5FEF8-CE3A-4E6E-B5F7-4600DCCBED95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF87F28-FC4F-4CF9-9C17-AC7D7F671F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tech Stack" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="389">
   <si>
     <t>NextJS</t>
   </si>
@@ -1291,12 +1291,144 @@
   <si>
     <t>Powerschool shares</t>
   </si>
+  <si>
+    <t>DynPro Documents</t>
+  </si>
+  <si>
+    <t>AWS Certified Solutions Architect Associate - SAA C03</t>
+  </si>
+  <si>
+    <t>Cloud Migration Approaches</t>
+  </si>
+  <si>
+    <t>Dev Ops</t>
+  </si>
+  <si>
+    <t>Dev Ops - CI, CD</t>
+  </si>
+  <si>
+    <t>Dev Ops - CI, CD Tools</t>
+  </si>
+  <si>
+    <t>Dev Ops - IAAC</t>
+  </si>
+  <si>
+    <t>AWS CloudFormation - Advantages</t>
+  </si>
+  <si>
+    <t>AWS CloudFormation - Intraduction</t>
+  </si>
+  <si>
+    <t>AWS CloudFormation - Terminology</t>
+  </si>
+  <si>
+    <t>AWS CloudFormation - Important template elements</t>
+  </si>
+  <si>
+    <t>AWS CloudFormation - Mapping Example</t>
+  </si>
+  <si>
+    <t>AWS CloudFormation - Remember</t>
+  </si>
+  <si>
+    <t>CloudFormation vs EBS</t>
+  </si>
+  <si>
+    <t>AWS OpsWorks - Configuration Management</t>
+  </si>
+  <si>
+    <t>Fault Tolerance</t>
+  </si>
+  <si>
+    <t>AWS Certification FAQ'S</t>
+  </si>
+  <si>
+    <t>Zero chance of Failure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWS Security Service </t>
+  </si>
+  <si>
+    <t>AWS Shield</t>
+  </si>
+  <si>
+    <t>AWS Shield Standard &amp; Advanced</t>
+  </si>
+  <si>
+    <t>AWS WAF - Web Application Firewall</t>
+  </si>
+  <si>
+    <t>AWS System Manager Parameter Store</t>
+  </si>
+  <si>
+    <t>AWS Secrets Manager</t>
+  </si>
+  <si>
+    <t>Amazon Macie</t>
+  </si>
+  <si>
+    <t>AWS Single Sign On</t>
+  </si>
+  <si>
+    <t>More security Services in AWS</t>
+  </si>
+  <si>
+    <t>More AWS Services</t>
+  </si>
+  <si>
+    <t>AWS Organisation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWS Organisations Features </t>
+  </si>
+  <si>
+    <t>AWS Resource Access Manager</t>
+  </si>
+  <si>
+    <t>One Enterprise - Many AWS accounts  -  AWS  Control Tower</t>
+  </si>
+  <si>
+    <t>AWS trusted advisor</t>
+  </si>
+  <si>
+    <t>AWS trusted advisor - Recommendations</t>
+  </si>
+  <si>
+    <t>AWS Service Quotas</t>
+  </si>
+  <si>
+    <t>AWS Directory Service</t>
+  </si>
+  <si>
+    <t>AWS Workspace</t>
+  </si>
+  <si>
+    <t>AWS Elemental Media Convert</t>
+  </si>
+  <si>
+    <t>Observability in AWS</t>
+  </si>
+  <si>
+    <t>More Management Services</t>
+  </si>
+  <si>
+    <t>AWS Proton</t>
+  </si>
+  <si>
+    <t>Machine Learning</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence - All around you</t>
+  </si>
+  <si>
+    <t>Architecture and Best Practice</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1376,6 +1508,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1428,7 +1567,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1459,6 +1598,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1967,7 +2110,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD904FA-0FAD-46CD-8773-AE594AFC6DAB}">
-  <dimension ref="B10:G321"/>
+  <dimension ref="B10:G380"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="8.7265625" customWidth="1"/>
@@ -3732,23 +3875,226 @@
       </c>
     </row>
     <row r="318" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F318" s="2" t="s">
+      <c r="F318" s="21" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="319" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F319" s="2" t="s">
+      <c r="F319" s="21" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="320" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F320" s="2" t="s">
+      <c r="F320" s="21" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="321" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F321" s="2" t="s">
+    <row r="321" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F321" s="21" t="s">
         <v>343</v>
+      </c>
+    </row>
+    <row r="322" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F322" s="2" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="325" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F325" s="2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="326" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F326" s="2" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="327" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F327" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="G327" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="328" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F328" s="2" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="329" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F329" s="2" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="330" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F330" s="2" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="331" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F331" s="2" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="332" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F332" s="2" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="333" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F333" s="2" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="334" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F334" s="2" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="335" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F335" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="336" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F336" s="2" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="339" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F339" s="2" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="342" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F342" s="2" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="343" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F343" s="2" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="344" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F344" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="345" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F345" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="346" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F346" s="2" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="347" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F347" s="2" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="348" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F348" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="349" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F349" s="2" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="350" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F350" s="2" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="355" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F355" s="2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="356" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F356" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="357" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F357" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="358" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F358" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="359" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F359" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="360" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F360" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="361" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F361" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="362" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F362" s="2" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="363" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F363" s="2" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="364" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F364" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="365" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F365" s="2" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="366" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F366" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="367" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F367" s="2" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="368" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F368" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="371" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F371" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="373" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F373" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="380" spans="6:6" x14ac:dyDescent="0.35">
+      <c r="F380" s="2" t="s">
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -3993,7 +4339,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr defaultRowHeight="18.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="98.7265625" style="4" customWidth="1"/>
@@ -4078,6 +4424,16 @@
     <row r="33" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A33" s="4" t="s">
         <v>344</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" s="20" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="20" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A35" s="4" t="s">
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -4090,55 +4446,63 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD312072-87FE-40B5-A445-1591614412BD}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="123.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>258</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>360</v>
+      </c>
+      <c r="B10" t="s">
+        <v>362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
File updated with aws
</commit_message>
<xml_diff>
--- a/Lookup.xlsx
+++ b/Lookup.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0201BB3E-1850-450E-9979-C1FC1EDC195C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{731D6759-7E23-4C95-B776-F849F9B399D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tech Stack" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="513">
   <si>
     <t>NextJS</t>
   </si>
@@ -1744,12 +1744,63 @@
   <si>
     <t>(Security / Networking / Data / ML)</t>
   </si>
+  <si>
+    <t>Service</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Amazon EC2</t>
+  </si>
+  <si>
+    <t>Run individual virtual servers</t>
+  </si>
+  <si>
+    <t>Amazon EMR</t>
+  </si>
+  <si>
+    <t>Amazon Athena</t>
+  </si>
+  <si>
+    <t>Run SQL queries directly on S3</t>
+  </si>
+  <si>
+    <t>Data warehouse analytics</t>
+  </si>
+  <si>
+    <t>Process huge datasets using clusters (With Hadoop)</t>
+  </si>
+  <si>
+    <t>Amazon DynamoDB</t>
+  </si>
+  <si>
+    <t>AWS Glue</t>
+  </si>
+  <si>
+    <t> - AWS Glue is a fully managed extract, transform, and load (ETL) service </t>
+  </si>
+  <si>
+    <t>is a fully managed NoSQL database service provided by AWS that stores and retrieves data with very low latency (very fast response time) and can automatically scale.</t>
+  </si>
+  <si>
+    <t>throttled</t>
+  </si>
+  <si>
+    <t>Samba 4</t>
+  </si>
+  <si>
+    <t>Too many requests are coming, so AWS temporarily reduces or blocks extra requests to protect the service.</t>
+  </si>
+  <si>
+    <t>aws glue DataBrew</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1836,6 +1887,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1888,7 +1954,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1925,6 +1991,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2431,11 +2504,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD904FA-0FAD-46CD-8773-AE594AFC6DAB}">
-  <dimension ref="B10:G502"/>
+  <dimension ref="B10:G526"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="8.7265625" customWidth="1"/>
     <col min="6" max="6" width="130.1796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="32.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="10" spans="6:6" ht="409.5" x14ac:dyDescent="0.55000000000000004">
@@ -4941,6 +5015,72 @@
     <row r="502" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F502" s="2" t="s">
         <v>488</v>
+      </c>
+    </row>
+    <row r="513" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F513" s="22" t="s">
+        <v>496</v>
+      </c>
+      <c r="G513" s="22" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="514" spans="6:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="F514" s="23" t="s">
+        <v>498</v>
+      </c>
+      <c r="G514" s="23" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="515" spans="6:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="F515" s="23" t="s">
+        <v>500</v>
+      </c>
+      <c r="G515" s="23" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="516" spans="6:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="F516" s="23" t="s">
+        <v>501</v>
+      </c>
+      <c r="G516" s="23" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="517" spans="6:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="F517" s="23" t="s">
+        <v>283</v>
+      </c>
+      <c r="G517" s="23" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="519" spans="6:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="F519" s="24" t="s">
+        <v>506</v>
+      </c>
+      <c r="G519" s="23" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="522" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F522" t="s">
+        <v>505</v>
+      </c>
+      <c r="G522" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="524" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F524" s="2" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="526" spans="6:7" x14ac:dyDescent="0.35">
+      <c r="F526" s="2" t="s">
+        <v>512</v>
       </c>
     </row>
   </sheetData>
@@ -5333,7 +5473,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD312072-87FE-40B5-A445-1591614412BD}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="123.36328125" customWidth="1"/>
@@ -5397,6 +5537,14 @@
         <v>489</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>509</v>
+      </c>
+      <c r="B12" t="s">
+        <v>511</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>